<commit_message>
fnal viernes 25 2025?
</commit_message>
<xml_diff>
--- a/originales/respuestas/2025/01. Calificadas/bucle p11/Agencia Distrital Para La Educación Superior, La Ciencia Y La Tecnología.xlsx
+++ b/originales/respuestas/2025/01. Calificadas/bucle p11/Agencia Distrital Para La Educación Superior, La Ciencia Y La Tecnología.xlsx
@@ -16,7 +16,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+  <si>
+    <t>Entidad</t>
+  </si>
   <si>
     <t>Tipo</t>
   </si>
@@ -212,7 +215,7 @@
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -451,101 +454,103 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="1"/>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E2" s="4">
         <v>4.20339688E8</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H2" s="6">
         <v>4.0</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J2" s="6">
         <v>4.0</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L2" s="6">
         <v>5.0</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="N2" s="6">
         <v>4.0</v>
       </c>
       <c r="O2" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P2" s="6">
         <v>1.0</v>

</xml_diff>